<commit_message>
actualiza acumulados 16/06/2026 19:02
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO-ARGELIA-(IED)-501_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO-ARGELIA-(IED)-501_CALIFICADO.xlsx
@@ -2313,10 +2313,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3321,10 +3325,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3570,10 +3578,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3819,10 +3831,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -4068,10 +4084,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -4317,10 +4337,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4819,10 +4843,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -5574,10 +5602,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -6329,10 +6361,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6578,10 +6614,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -11618,10 +11658,14 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -12622,10 +12666,14 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -12871,10 +12919,14 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -13120,10 +13172,14 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -13369,10 +13425,14 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -13618,10 +13678,14 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -14120,10 +14184,14 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -14875,10 +14943,14 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -15630,10 +15702,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -15879,10 +15955,14 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>111001100084</t>
+          <t>111001100064</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">

</xml_diff>